<commit_message>
Implemented new prompt, batch Claude, linear regression model for AI adoption score.
</commit_message>
<xml_diff>
--- a/Batch_A_Report.xlsx
+++ b/Batch_A_Report.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F52"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -453,7 +453,7 @@
         <v>6281</v>
       </c>
       <c r="B2" t="n">
-        <v>0.03675</v>
+        <v>0.0024</v>
       </c>
       <c r="C2" t="n">
         <v>1632</v>
@@ -525,7 +525,7 @@
         <v>50863</v>
       </c>
       <c r="B5" t="n">
-        <v>5.524925000000001</v>
+        <v>3.35222</v>
       </c>
       <c r="C5" t="n">
         <v>6008</v>
@@ -621,7 +621,7 @@
         <v>106040</v>
       </c>
       <c r="B9" t="n">
-        <v>0.1716</v>
+        <v>0.0351</v>
       </c>
       <c r="C9" t="n">
         <v>11399</v>
@@ -717,7 +717,7 @@
         <v>723125</v>
       </c>
       <c r="B13" t="n">
-        <v>2.2212</v>
+        <v>1.33485</v>
       </c>
       <c r="C13" t="n">
         <v>7343</v>
@@ -765,7 +765,7 @@
         <v>789019</v>
       </c>
       <c r="B15" t="n">
-        <v>12.683135</v>
+        <v>7.670036500000001</v>
       </c>
       <c r="C15" t="n">
         <v>12141</v>
@@ -786,113 +786,113 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>792130</v>
+        <v>794323</v>
       </c>
       <c r="B16" t="n">
-        <v>1.904905</v>
+        <v>0</v>
       </c>
       <c r="C16" t="n">
-        <v>25320</v>
+        <v>13440</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>DATAWATCH CORP</t>
+          <t>LEVEL 3 COMMUNICATIONS INC</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0</v>
+        <v>0.0006079027079977</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>511210</t>
+          <t>519130</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>794323</v>
+        <v>796343</v>
       </c>
       <c r="B17" t="n">
-        <v>0</v>
+        <v>2.03946</v>
       </c>
       <c r="C17" t="n">
-        <v>13440</v>
+        <v>12540</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>LEVEL 3 COMMUNICATIONS INC</t>
+          <t>ADOBE SYSTEMS INC</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.0006079027079977</v>
+        <v>0.0239260476082563</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>519130</t>
+          <t>451110</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>796343</v>
+        <v>798354</v>
       </c>
       <c r="B18" t="n">
-        <v>2.822072</v>
+        <v>0.1728</v>
       </c>
       <c r="C18" t="n">
-        <v>12540</v>
+        <v>12635</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>ADOBE SYSTEMS INC</t>
+          <t>FISERV INC</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>0.0239260476082563</v>
+        <v>0.0002362949016969</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>451110</t>
+          <t>334111</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>798354</v>
+        <v>814547</v>
       </c>
       <c r="B19" t="n">
-        <v>0.126225</v>
+        <v>15.547695</v>
       </c>
       <c r="C19" t="n">
-        <v>12635</v>
+        <v>13824</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>FISERV INC</t>
+          <t>FAIR ISAAC CORP</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>0.0002362949016969</v>
+        <v>0</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>334111</t>
+          <t>541512</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>814547</v>
+        <v>828146</v>
       </c>
       <c r="B20" t="n">
-        <v>11.7016</v>
+        <v>0</v>
       </c>
       <c r="C20" t="n">
-        <v>13824</v>
+        <v>28374</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>FAIR ISAAC CORP</t>
+          <t>INTERLINK ELECTRONICS</t>
         </is>
       </c>
       <c r="E20" t="n">
@@ -900,23 +900,23 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>541512</t>
+          <t>518210</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>828146</v>
+        <v>849547</v>
       </c>
       <c r="B21" t="n">
         <v>0</v>
       </c>
       <c r="C21" t="n">
-        <v>28374</v>
+        <v>26012</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>INTERLINK ELECTRONICS</t>
+          <t>BLACK BOX CORP</t>
         </is>
       </c>
       <c r="E21" t="n">
@@ -924,95 +924,95 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>518210</t>
+          <t>511210</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>849547</v>
+        <v>857005</v>
       </c>
       <c r="B22" t="n">
-        <v>0</v>
+        <v>2.45916</v>
       </c>
       <c r="C22" t="n">
-        <v>26012</v>
+        <v>18699</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>BLACK BOX CORP</t>
+          <t>PARAMETRIC TECHNOLOGY CORP</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>0</v>
+        <v>0.0051993066444993</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>511210</t>
+          <t>334210</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>857005</v>
+        <v>858877</v>
       </c>
       <c r="B23" t="n">
-        <v>2.34657</v>
+        <v>3.08902</v>
       </c>
       <c r="C23" t="n">
-        <v>18699</v>
+        <v>20779</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>PARAMETRIC TECHNOLOGY CORP</t>
+          <t>CISCO SYSTEMS INC</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>0.0051993066444993</v>
+        <v>0.0061595761217176</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>334210</t>
+          <t>.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>858877</v>
+        <v>866729</v>
       </c>
       <c r="B24" t="n">
-        <v>3.46575</v>
+        <v>0</v>
       </c>
       <c r="C24" t="n">
-        <v>20779</v>
+        <v>5349</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>CISCO SYSTEMS INC</t>
+          <t>GROLIER INC</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>0.0061595761217176</v>
+        <v>0</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>519130</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>866729</v>
+        <v>882835</v>
       </c>
       <c r="B25" t="n">
         <v>0</v>
       </c>
       <c r="C25" t="n">
-        <v>5349</v>
+        <v>64423</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>GROLIER INC</t>
+          <t>DELTEK SYSTEMS INC</t>
         </is>
       </c>
       <c r="E25" t="n">
@@ -1020,23 +1020,23 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>519130</t>
+          <t>334413</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>882835</v>
+        <v>884144</v>
       </c>
       <c r="B26" t="n">
-        <v>0</v>
+        <v>0.0102</v>
       </c>
       <c r="C26" t="n">
-        <v>64423</v>
+        <v>25138</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>DELTEK SYSTEMS INC</t>
+          <t>FORGENT NETWORKS INC</t>
         </is>
       </c>
       <c r="E26" t="n">
@@ -1044,95 +1044,95 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>334413</t>
+          <t>541512</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>884144</v>
+        <v>896841</v>
       </c>
       <c r="B27" t="n">
-        <v>0.006000000000000002</v>
+        <v>0</v>
       </c>
       <c r="C27" t="n">
-        <v>25138</v>
+        <v>27925</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>FORGENT NETWORKS INC</t>
+          <t>AVID TECHNOLOGY INC</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>0</v>
+        <v>0.005167958792299</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>541512</t>
+          <t>334220</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>896841</v>
+        <v>896878</v>
       </c>
       <c r="B28" t="n">
-        <v>0</v>
+        <v>1.30682</v>
       </c>
       <c r="C28" t="n">
-        <v>27925</v>
+        <v>27928</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>AVID TECHNOLOGY INC</t>
+          <t>INTUIT INC</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>0.005167958792299</v>
+        <v>0.0137825421988964</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>334220</t>
+          <t>337127</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>896878</v>
+        <v>903651</v>
       </c>
       <c r="B29" t="n">
-        <v>2.021495</v>
+        <v>0.2366</v>
       </c>
       <c r="C29" t="n">
-        <v>27928</v>
+        <v>28717</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>INTUIT INC</t>
+          <t>INNODATA ISOGEN INC</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>0.0137825421988964</v>
+        <v>0</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>337127</t>
+          <t>519130</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>903651</v>
+        <v>909494</v>
       </c>
       <c r="B30" t="n">
-        <v>0.425425</v>
+        <v>0</v>
       </c>
       <c r="C30" t="n">
-        <v>28717</v>
+        <v>62723</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>INNODATA ISOGEN INC</t>
+          <t>TUCOWS INC</t>
         </is>
       </c>
       <c r="E30" t="n">
@@ -1140,23 +1140,23 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>519130</t>
+          <t>334413</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>909494</v>
+        <v>912093</v>
       </c>
       <c r="B31" t="n">
         <v>0</v>
       </c>
       <c r="C31" t="n">
-        <v>62723</v>
+        <v>29241</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>TUCOWS INC</t>
+          <t>JDS UNIPHASE CORP</t>
         </is>
       </c>
       <c r="E31" t="n">
@@ -1170,65 +1170,65 @@
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>912093</v>
+        <v>935036</v>
       </c>
       <c r="B32" t="n">
-        <v>0</v>
+        <v>0.7289999999999999</v>
       </c>
       <c r="C32" t="n">
-        <v>29241</v>
+        <v>31564</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>JDS UNIPHASE CORP</t>
+          <t>TRNSACTN SYS ARCHTCTS  -CL A</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>0</v>
+        <v>0.0013386880746111</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>334413</t>
+          <t>518210</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>935036</v>
+        <v>943034</v>
       </c>
       <c r="B33" t="n">
-        <v>0.8747999999999999</v>
+        <v>0</v>
       </c>
       <c r="C33" t="n">
-        <v>31564</v>
+        <v>31775</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>TRNSACTN SYS ARCHTCTS  -CL A</t>
+          <t>IMAGE SENSING SYSTEMS INC</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>0.0013386880746111</v>
+        <v>0</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>518210</t>
+          <t>334419</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>943034</v>
+        <v>1014111</v>
       </c>
       <c r="B34" t="n">
         <v>0</v>
       </c>
       <c r="C34" t="n">
-        <v>31775</v>
+        <v>7244</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>IMAGE SENSING SYSTEMS INC</t>
+          <t>MEMOREX CORP</t>
         </is>
       </c>
       <c r="E34" t="n">
@@ -1236,95 +1236,95 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>334419</t>
+          <t>51121</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>1014111</v>
+        <v>1018724</v>
       </c>
       <c r="B35" t="n">
         <v>0</v>
       </c>
       <c r="C35" t="n">
-        <v>7244</v>
+        <v>64768</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>MEMOREX CORP</t>
+          <t>AMAZON.COM INC</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>0</v>
+        <v>0.0122375879436731</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>51121</t>
+          <t>.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>1018724</v>
+        <v>1024478</v>
       </c>
       <c r="B36" t="n">
         <v>0</v>
       </c>
       <c r="C36" t="n">
-        <v>64768</v>
+        <v>9203</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>AMAZON.COM INC</t>
+          <t>ROCKWELL AUTOMATION</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>0.0122375879436731</v>
+        <v>0.0007662835414521</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>541512</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>1024478</v>
+        <v>1029744</v>
       </c>
       <c r="B37" t="n">
         <v>0</v>
       </c>
       <c r="C37" t="n">
-        <v>9203</v>
+        <v>109186</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>ROCKWELL AUTOMATION</t>
+          <t>SONIC FOUNDRY INC</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>0.0007662835414521</v>
+        <v>0</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>541512</t>
+          <t>334119</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>1029744</v>
+        <v>1036188</v>
       </c>
       <c r="B38" t="n">
-        <v>0</v>
+        <v>0.1072</v>
       </c>
       <c r="C38" t="n">
-        <v>109186</v>
+        <v>65226</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>SONIC FOUNDRY INC</t>
+          <t>QAD INC</t>
         </is>
       </c>
       <c r="E38" t="n">
@@ -1332,23 +1332,23 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>334119</t>
+          <t>511210</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>1036188</v>
+        <v>1038222</v>
       </c>
       <c r="B39" t="n">
-        <v>0.277725</v>
+        <v>0</v>
       </c>
       <c r="C39" t="n">
-        <v>65226</v>
+        <v>64850</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>QAD INC</t>
+          <t>REIS INC</t>
         </is>
       </c>
       <c r="E39" t="n">
@@ -1356,167 +1356,167 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>511210</t>
+          <t>519130</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>1038222</v>
+        <v>1065280</v>
       </c>
       <c r="B40" t="n">
         <v>0</v>
       </c>
       <c r="C40" t="n">
-        <v>64850</v>
+        <v>147579</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>REIS INC</t>
+          <t>NETFLIX INC</t>
         </is>
       </c>
       <c r="E40" t="n">
-        <v>0</v>
+        <v>0.0133382733911275</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>519130</t>
+          <t>332721</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>1065280</v>
+        <v>1078099</v>
       </c>
       <c r="B41" t="n">
         <v>0</v>
       </c>
       <c r="C41" t="n">
-        <v>147579</v>
+        <v>121662</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>NETFLIX INC</t>
+          <t>QUEPASA CORP</t>
         </is>
       </c>
       <c r="E41" t="n">
-        <v>0.0133382733911275</v>
+        <v>0</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>332721</t>
+          <t>541512</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>1078099</v>
+        <v>1087423</v>
       </c>
       <c r="B42" t="n">
         <v>0</v>
       </c>
       <c r="C42" t="n">
-        <v>121662</v>
+        <v>122841</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>QUEPASA CORP</t>
+          <t>RED HAT INC</t>
         </is>
       </c>
       <c r="E42" t="n">
-        <v>0</v>
+        <v>0.0047281323932111</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>541512</t>
+          <t>334119</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>1087423</v>
+        <v>1108524</v>
       </c>
       <c r="B43" t="n">
-        <v>0</v>
+        <v>2.991785</v>
       </c>
       <c r="C43" t="n">
-        <v>122841</v>
+        <v>157855</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>RED HAT INC</t>
+          <t>SALESFORCE.COM INC</t>
         </is>
       </c>
       <c r="E43" t="n">
-        <v>0.0047281323932111</v>
+        <v>0.0081739416345953</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>334119</t>
+          <t>325414</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>1108524</v>
+        <v>1130713</v>
       </c>
       <c r="B44" t="n">
-        <v>6.219109</v>
+        <v>0.1998</v>
       </c>
       <c r="C44" t="n">
-        <v>157855</v>
+        <v>147868</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>SALESFORCE.COM INC</t>
+          <t>OVERSTOCK.COM INC</t>
         </is>
       </c>
       <c r="E44" t="n">
-        <v>0.0081739416345953</v>
+        <v>0.015358361415565</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>325414</t>
+          <t>511210</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>1130713</v>
+        <v>1157817</v>
       </c>
       <c r="B45" t="n">
-        <v>0.37315</v>
+        <v>0</v>
       </c>
       <c r="C45" t="n">
-        <v>147868</v>
+        <v>149360</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>OVERSTOCK.COM INC</t>
+          <t>HOSTING SITE NETWORK INC</t>
         </is>
       </c>
       <c r="E45" t="n">
-        <v>0.015358361415565</v>
+        <v>0</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>511210</t>
+          <t>334413</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>1157817</v>
+        <v>1296445</v>
       </c>
       <c r="B46" t="n">
         <v>0</v>
       </c>
       <c r="C46" t="n">
-        <v>149360</v>
+        <v>160913</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>HOSTING SITE NETWORK INC</t>
+          <t>ORMAT TECHNOLOGIES INC</t>
         </is>
       </c>
       <c r="E46" t="n">
@@ -1524,71 +1524,71 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>334413</t>
+          <t>511210</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>1296445</v>
+        <v>1341439</v>
       </c>
       <c r="B47" t="n">
-        <v>0</v>
+        <v>1.33722</v>
       </c>
       <c r="C47" t="n">
-        <v>160913</v>
+        <v>12142</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>ORMAT TECHNOLOGIES INC</t>
+          <t>ORACLE CORP</t>
         </is>
       </c>
       <c r="E47" t="n">
-        <v>0</v>
+        <v>0.0071220458485186</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>511210</t>
+          <t>561990</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>1341439</v>
+        <v>1561880</v>
       </c>
       <c r="B48" t="n">
-        <v>1.86171</v>
+        <v>0</v>
       </c>
       <c r="C48" t="n">
-        <v>12142</v>
+        <v>114242</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>ORACLE CORP</t>
+          <t>WHITNEY INFORMATION NET INC</t>
         </is>
       </c>
       <c r="E48" t="n">
-        <v>0.0071220458485186</v>
+        <v>0</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>561990</t>
+          <t>541519</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>1561880</v>
+        <v>1633917</v>
       </c>
       <c r="B49" t="n">
         <v>0</v>
       </c>
       <c r="C49" t="n">
-        <v>114242</v>
+        <v>145471</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>WHITNEY INFORMATION NET INC</t>
+          <t>PAYPAL INC</t>
         </is>
       </c>
       <c r="E49" t="n">
@@ -1596,77 +1596,53 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>541519</t>
+          <t>334310</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>1633917</v>
+        <v>1645494</v>
       </c>
       <c r="B50" t="n">
         <v>0</v>
       </c>
       <c r="C50" t="n">
-        <v>145471</v>
+        <v>28853</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>PAYPAL INC</t>
+          <t>ARRIS GROUP INC</t>
         </is>
       </c>
       <c r="E50" t="n">
-        <v>0</v>
+        <v>0.0011198208667337</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>334310</t>
+          <t>511210</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>1645494</v>
+        <v>1652044</v>
       </c>
       <c r="B51" t="n">
-        <v>0</v>
+        <v>3.355939999999999</v>
       </c>
       <c r="C51" t="n">
-        <v>28853</v>
+        <v>160329</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>ARRIS GROUP INC</t>
+          <t>GOOGLE INC</t>
         </is>
       </c>
       <c r="E51" t="n">
-        <v>0.0011198208667337</v>
+        <v>0.0297704450786113</v>
       </c>
       <c r="F51" t="inlineStr">
-        <is>
-          <t>511210</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="n">
-        <v>1652044</v>
-      </c>
-      <c r="B52" t="n">
-        <v>4.041088</v>
-      </c>
-      <c r="C52" t="n">
-        <v>160329</v>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>GOOGLE INC</t>
-        </is>
-      </c>
-      <c r="E52" t="n">
-        <v>0.0297704450786113</v>
-      </c>
-      <c r="F52" t="inlineStr">
         <is>
           <t>334111</t>
         </is>

</xml_diff>